<commit_message>
The UI for general  notice is fucked up, use similar to holiday notice a
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhatt\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{922CFFD7-E3DC-4226-B42C-37E6EF529CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF4E53E-DB06-4CDA-997F-004A1F2F8152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{4F6E8338-436D-42B2-9008-EDFC726C3FE2}"/>
   </bookViews>
   <sheets>
-    <sheet name="Notices" sheetId="1" r:id="rId1"/>
-    <sheet name="Results" sheetId="2" r:id="rId2"/>
+    <sheet name="GeneralNotices" sheetId="4" r:id="rId1"/>
+    <sheet name="Holidays" sheetId="3" r:id="rId2"/>
+    <sheet name="ExamNotices" sheetId="1" r:id="rId3"/>
+    <sheet name="Results" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t>title</t>
   </si>
@@ -79,13 +81,58 @@
   </si>
   <si>
     <t>https://bbhatt.com.np</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>details</t>
+  </si>
+  <si>
+    <t>summary</t>
+  </si>
+  <si>
+    <t>icon</t>
+  </si>
+  <si>
+    <t>Mock Data 1</t>
+  </si>
+  <si>
+    <t>Mock Data 2</t>
+  </si>
+  <si>
+    <t>Mock Data 3</t>
+  </si>
+  <si>
+    <t>Bell</t>
+  </si>
+  <si>
+    <t>FileText</t>
+  </si>
+  <si>
+    <t>…</t>
+  </si>
+  <si>
+    <t>2082-02-02 to 2082-02-03</t>
+  </si>
+  <si>
+    <t>2082-02-02 to 2082-02-04</t>
+  </si>
+  <si>
+    <t>2082-02-02 to 2082-02-05</t>
+  </si>
+  <si>
+    <t>Calendar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="171" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -97,6 +144,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -125,8 +178,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -461,18 +514,148 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D14FC3B3-2AAB-4D6A-9BA6-A195DDD1C4A1}">
-  <dimension ref="A1:D2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{820D46FA-ACC3-4246-8664-7204E505C772}">
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="2">
+        <v>66782</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2">
+        <v>66783</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2">
+        <v>66784</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13A85314-165E-4808-847D-10018C6DFF73}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D14FC3B3-2AAB-4D6A-9BA6-A195DDD1C4A1}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -486,25 +669,54 @@
       <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>66782</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2">
+        <v>66783</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2">
+        <v>66784</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{CE314454-4769-4F63-A0BB-91C460B4A6A0}"/>
+    <hyperlink ref="D3:D4" r:id="rId2" display="https://bbhatt.com.np" xr:uid="{1ECD11F9-3B95-49F2-9071-6DD1FE081E54}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC53C596-5529-4790-AB27-E412B3A7F756}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Use a better Ui for the result check model
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhatt\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF4E53E-DB06-4CDA-997F-004A1F2F8152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FC2F48-7631-420C-AB2C-2DC8A149E6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{4F6E8338-436D-42B2-9008-EDFC726C3FE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="3" xr2:uid="{4F6E8338-436D-42B2-9008-EDFC726C3FE2}"/>
   </bookViews>
   <sheets>
     <sheet name="GeneralNotices" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
   <si>
     <t>title</t>
   </si>
@@ -123,6 +123,30 @@
   </si>
   <si>
     <t>Calendar</t>
+  </si>
+  <si>
+    <t>Mock Data 4</t>
+  </si>
+  <si>
+    <t>Mock Data 5</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>DOB</t>
   </si>
 </sst>
 </file>
@@ -718,13 +742,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC53C596-5529-4790-AB27-E412B3A7F756}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -732,33 +757,120 @@
         <v>5</v>
       </c>
       <c r="C1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>83035</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2">
+        <v>60411</v>
+      </c>
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>9.6999999999999993</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>11</v>
       </c>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3">
+        <v>83036</v>
+      </c>
+      <c r="C3" s="2">
+        <v>60412</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3">
+        <v>5.3</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <v>83037</v>
+      </c>
+      <c r="C4" s="2">
+        <v>60413</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5">
+        <v>83038</v>
+      </c>
+      <c r="C5" s="2">
+        <v>60414</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5">
+        <v>3.3</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6">
+        <v>83039</v>
+      </c>
+      <c r="C6" s="2">
+        <v>60415</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
The data isn't sowing after checking result, its only expanding the resu
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhatt\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FC2F48-7631-420C-AB2C-2DC8A149E6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA528C63-066B-4DF3-86AD-2F46F16B2140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="3" xr2:uid="{4F6E8338-436D-42B2-9008-EDFC726C3FE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{4F6E8338-436D-42B2-9008-EDFC726C3FE2}"/>
   </bookViews>
   <sheets>
     <sheet name="GeneralNotices" sheetId="4" r:id="rId1"/>
@@ -113,15 +113,6 @@
     <t>…</t>
   </si>
   <si>
-    <t>2082-02-02 to 2082-02-03</t>
-  </si>
-  <si>
-    <t>2082-02-02 to 2082-02-04</t>
-  </si>
-  <si>
-    <t>2082-02-02 to 2082-02-05</t>
-  </si>
-  <si>
     <t>Calendar</t>
   </si>
   <si>
@@ -147,6 +138,15 @@
   </si>
   <si>
     <t>DOB</t>
+  </si>
+  <si>
+    <t>4 to 8 Falugun, 2082</t>
+  </si>
+  <si>
+    <t>5 to 8 Falugun, 2082</t>
+  </si>
+  <si>
+    <t>6 to 8 Falugun, 2082</t>
   </si>
 </sst>
 </file>
@@ -599,7 +599,7 @@
         <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -633,7 +633,7 @@
         <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
         <v>23</v>
@@ -644,7 +644,7 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
         <v>23</v>
@@ -655,7 +655,7 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
@@ -757,7 +757,7 @@
         <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
@@ -800,13 +800,13 @@
         <v>60412</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E3">
         <v>5.3</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -820,18 +820,18 @@
         <v>60413</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E4">
         <v>2.2000000000000002</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>83038</v>
@@ -840,7 +840,7 @@
         <v>60414</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E5">
         <v>3.3</v>
@@ -851,7 +851,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B6">
         <v>83039</v>
@@ -860,7 +860,7 @@
         <v>60415</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E6">
         <v>2.2000000000000002</v>

</xml_diff>

<commit_message>
Use a modern, sleek and better professional UI, also use Facilities text
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhatt\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA528C63-066B-4DF3-86AD-2F46F16B2140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F75F7D18-D8F3-4A92-8C11-ECF7976B5315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{4F6E8338-436D-42B2-9008-EDFC726C3FE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{4F6E8338-436D-42B2-9008-EDFC726C3FE2}"/>
   </bookViews>
   <sheets>
     <sheet name="GeneralNotices" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="37">
   <si>
     <t>title</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>6 to 8 Falugun, 2082</t>
+  </si>
+  <si>
+    <t>MockData 1 detailed description …</t>
   </si>
 </sst>
 </file>
@@ -154,7 +157,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="171" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -203,7 +206,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -539,14 +542,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{820D46FA-ACC3-4246-8664-7204E505C772}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -559,8 +562,11 @@
       <c r="D1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -573,8 +579,11 @@
       <c r="D2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -587,8 +596,11 @@
       <c r="D3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -600,6 +612,9 @@
       </c>
       <c r="D4" t="s">
         <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Try fixing this error: `Console Error: Only plain objects can be passed
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="GeneralNotices" sheetId="1" r:id="rId1"/>
     <sheet name="Holidays" sheetId="2" r:id="rId2"/>
@@ -536,7 +536,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -556,7 +556,7 @@
       <c r="A2" t="str">
         <v>Mock Data</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="str">
         <v>66782</v>
       </c>
       <c r="C2" t="str">
@@ -570,7 +570,7 @@
       <c r="A3" t="str">
         <v>Mock Data</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="str">
         <v>66783</v>
       </c>
       <c r="C3" t="str">
@@ -584,7 +584,7 @@
       <c r="A4" t="str">
         <v>Mock Data</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="str">
         <v>66784</v>
       </c>
       <c r="C4" t="str">
@@ -594,15 +594,23 @@
         <v>https://bbhatt.com.np</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Mock Data</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2082-05-24</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Routine</v>
+      </c>
+      <c r="D5" t="str">
+        <v>https://bbhatt.com.np</v>
+      </c>
+    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
-    <hyperlink ref="D3" r:id="rId2"/>
-    <hyperlink ref="D4" r:id="rId3"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Where is the logout buttons?
Also for fail, the grade is NG
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -643,17 +643,17 @@
       <c r="A2" t="str">
         <v>Mock Data 1</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="str">
         <v>83035</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="str">
         <v>60411</v>
       </c>
       <c r="D2" t="str">
         <v>A+</v>
       </c>
-      <c r="E2">
-        <v>9.7</v>
+      <c r="E2" t="str">
+        <v>4</v>
       </c>
       <c r="F2" t="str">
         <v>Pass</v>
@@ -663,56 +663,56 @@
       <c r="A3" t="str">
         <v>Mock Data 2</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="str">
         <v>83036</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="str">
         <v>60412</v>
       </c>
       <c r="D3" t="str">
-        <v>A</v>
-      </c>
-      <c r="E3">
-        <v>5.3</v>
+        <v>B+</v>
+      </c>
+      <c r="E3" t="str">
+        <v>3</v>
       </c>
       <c r="F3" t="str">
-        <v>Fail</v>
+        <v>Pass</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>Mock Data 3</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="str">
         <v>83037</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="str">
         <v>60413</v>
       </c>
       <c r="D4" t="str">
-        <v>B</v>
-      </c>
-      <c r="E4">
-        <v>2.2</v>
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
       </c>
       <c r="F4" t="str">
-        <v>Fail</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
         <v>Mock Data 4</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="str">
         <v>83038</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="str">
         <v>60414</v>
       </c>
       <c r="D5" t="str">
         <v>C</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="str">
         <v>3.3</v>
       </c>
       <c r="F5" t="str">
@@ -723,16 +723,16 @@
       <c r="A6" t="str">
         <v>Mock Data 5</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="str">
         <v>83039</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="str">
         <v>60415</v>
       </c>
       <c r="D6" t="str">
         <v>B+</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="str">
         <v>2.2</v>
       </c>
       <c r="F6" t="str">
@@ -740,7 +740,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
One thing after deleting the rows  it shouldn't ask for save changes, de
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,16 +422,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Mock Data 1</v>
-      </c>
-      <c r="B2">
-        <v>66782</v>
+        <v>Mock Data 2</v>
+      </c>
+      <c r="B2" t="str">
+        <v>66783</v>
       </c>
       <c r="C2" t="str">
-        <v>…ello</v>
+        <v>…</v>
       </c>
       <c r="D2" t="str">
-        <v>Bell</v>
+        <v>FileText</v>
       </c>
       <c r="E2" t="str">
         <v>MockData 1 detailed description …</v>
@@ -439,48 +439,31 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Mock Data 2</v>
-      </c>
-      <c r="B3">
-        <v>66783</v>
+        <v>Mock Data 3</v>
+      </c>
+      <c r="B3" t="str">
+        <v>66784</v>
       </c>
       <c r="C3" t="str">
         <v>…</v>
       </c>
       <c r="D3" t="str">
-        <v>FileText</v>
+        <v>Calendar</v>
       </c>
       <c r="E3" t="str">
         <v>MockData 1 detailed description …</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Mock Data 3</v>
-      </c>
-      <c r="B4">
-        <v>66784</v>
-      </c>
-      <c r="C4" t="str">
-        <v>…</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Calendar</v>
-      </c>
-      <c r="E4" t="str">
-        <v>MockData 1 detailed description …</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -493,43 +476,9 @@
         <v>details</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Mock Data 1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>4 to 8 Falugun, 2082</v>
-      </c>
-      <c r="C2" t="str">
-        <v>…</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Mock Data 2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>5 to 8 Falugun, 2082</v>
-      </c>
-      <c r="C3" t="str">
-        <v>…</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Mock Data 3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>6 to 8 Falugun, 2082</v>
-      </c>
-      <c r="C4" t="str">
-        <v>…</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Try fixing this error: `Runtime Error: A <Select.Item /> must have a val
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,41 +422,24 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Mock Data 2</v>
+        <v>ANNUAL FUNCTION 2082</v>
       </c>
       <c r="B2" t="str">
-        <v>66783</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>…</v>
+        <v>We are excited to announce the Annual Function 2082, a day dedicated to celebrating student talent and academic excellence. All students and staff are invited to join the festivities and honor our collective achievements.</v>
       </c>
       <c r="D2" t="str">
-        <v>FileText</v>
+        <v>Bell</v>
       </c>
       <c r="E2" t="str">
-        <v>MockData 1 detailed description …</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Mock Data 3</v>
-      </c>
-      <c r="B3" t="str">
-        <v>66784</v>
-      </c>
-      <c r="C3" t="str">
-        <v>…</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Calendar</v>
-      </c>
-      <c r="E3" t="str">
-        <v>MockData 1 detailed description …</v>
+        <v>This notice serves to inform all students, faculty, and staff that the college’s most anticipated event of the year—the Annual Function—is scheduled for Falgun 07, 2082. This day is dedicated to celebrating our academic achievements, showcasing student talent, and fostering community spirit. Classes will remain suspended on this day to allow full participation in the festivities.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -485,7 +468,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -501,72 +484,16 @@
         <v>link</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Mock Data</v>
-      </c>
-      <c r="B2" t="str">
-        <v>66782</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Routine</v>
-      </c>
-      <c r="D2" t="str">
-        <v>https://bbhatt.com.np</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Mock Data</v>
-      </c>
-      <c r="B3" t="str">
-        <v>66783</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Routine</v>
-      </c>
-      <c r="D3" t="str">
-        <v>https://bbhatt.com.np</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Mock Data</v>
-      </c>
-      <c r="B4" t="str">
-        <v>66784</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Routine</v>
-      </c>
-      <c r="D4" t="str">
-        <v>https://bbhatt.com.np</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Mock Data</v>
-      </c>
-      <c r="B5" t="str">
-        <v>2082-05-24</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Routine</v>
-      </c>
-      <c r="D5" t="str">
-        <v>https://bbhatt.com.np</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -588,109 +515,9 @@
         <v>Remarks</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Mock Data 1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>83035</v>
-      </c>
-      <c r="C2" t="str">
-        <v>60411</v>
-      </c>
-      <c r="D2" t="str">
-        <v>A+</v>
-      </c>
-      <c r="E2" t="str">
-        <v>4</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Pass</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Mock Data 2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>83036</v>
-      </c>
-      <c r="C3" t="str">
-        <v>60412</v>
-      </c>
-      <c r="D3" t="str">
-        <v>B+</v>
-      </c>
-      <c r="E3" t="str">
-        <v>3</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Pass</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Mock Data 3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>83037</v>
-      </c>
-      <c r="C4" t="str">
-        <v>60413</v>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Mock Data 4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>83038</v>
-      </c>
-      <c r="C5" t="str">
-        <v>60414</v>
-      </c>
-      <c r="D5" t="str">
-        <v>C</v>
-      </c>
-      <c r="E5" t="str">
-        <v>3.3</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Pass</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Mock Data 5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>83039</v>
-      </c>
-      <c r="C6" t="str">
-        <v>60415</v>
-      </c>
-      <c r="D6" t="str">
-        <v>B+</v>
-      </c>
-      <c r="E6" t="str">
-        <v>2.2</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Pass</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update the tab (sheet) switcing texts to General, Holiday, Exams & Resul
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -68,9 +68,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,84 +420,16 @@
         <v>details</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Mock Data 1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>2082-11-02</v>
-      </c>
-      <c r="C2" t="str">
-        <v>…</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Bell</v>
-      </c>
-      <c r="E2" t="str">
-        <v>MockData 1 detailed description …</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Mock Data 2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2082-11-03</v>
-      </c>
-      <c r="C3" t="str">
-        <v>…</v>
-      </c>
-      <c r="D3" t="str">
-        <v>FileText</v>
-      </c>
-      <c r="E3" t="str">
-        <v>MockData 1 detailed description …</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Mock Data 3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>2082-11-04</v>
-      </c>
-      <c r="C4" t="str">
-        <v>…</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Calendar</v>
-      </c>
-      <c r="E4" t="str">
-        <v>MockData 1 detailed description …</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Annuals Fo</v>
-      </c>
-      <c r="B5" t="str">
-        <v>387293</v>
-      </c>
-      <c r="C5" t="str">
-        <v>3987</v>
-      </c>
-      <c r="D5" t="str">
-        <v>dc</v>
-      </c>
-      <c r="E5" t="str">
-        <v>3279872</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -511,50 +442,16 @@
         <v>details</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Mock Data 1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>4 to 8 Falugun, 2082</v>
-      </c>
-      <c r="C2" t="str">
-        <v>…</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Mock Data 2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>5 to 8 Falugun, 2082</v>
-      </c>
-      <c r="C3" t="str">
-        <v>…</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Mock Data 3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>6 to 8 Falugun, 2082</v>
-      </c>
-      <c r="C4" t="str">
-        <v>…</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -570,64 +467,16 @@
         <v>link</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Mock Data</v>
-      </c>
-      <c r="B2" s="1">
-        <v>66782</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Routine</v>
-      </c>
-      <c r="D2" t="str">
-        <v>https://bbhatt.com.np</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Mock Data</v>
-      </c>
-      <c r="B3" s="1">
-        <v>66783</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Routine</v>
-      </c>
-      <c r="D3" t="str">
-        <v>https://bbhatt.com.np</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Mock Data</v>
-      </c>
-      <c r="B4" s="1">
-        <v>66784</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Routine</v>
-      </c>
-      <c r="D4" t="str">
-        <v>https://bbhatt.com.np</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
-    <hyperlink ref="D3" r:id="rId2"/>
-    <hyperlink ref="D4" r:id="rId3"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -649,110 +498,9 @@
         <v>Remarks</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Mock Data 1</v>
-      </c>
-      <c r="B2">
-        <v>83035</v>
-      </c>
-      <c r="C2" s="1">
-        <v>60411</v>
-      </c>
-      <c r="D2" t="str">
-        <v>A+</v>
-      </c>
-      <c r="E2">
-        <v>9.7</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Pass</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Mock Data 2</v>
-      </c>
-      <c r="B3">
-        <v>83036</v>
-      </c>
-      <c r="C3" s="1">
-        <v>60412</v>
-      </c>
-      <c r="D3" t="str">
-        <v>A</v>
-      </c>
-      <c r="E3">
-        <v>5.3</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Fail</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Mock Data 3</v>
-      </c>
-      <c r="B4">
-        <v>83037</v>
-      </c>
-      <c r="C4" s="1">
-        <v>60413</v>
-      </c>
-      <c r="D4" t="str">
-        <v>B</v>
-      </c>
-      <c r="E4">
-        <v>2.2</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Fail</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Mock Data 4</v>
-      </c>
-      <c r="B5">
-        <v>83038</v>
-      </c>
-      <c r="C5" s="1">
-        <v>60414</v>
-      </c>
-      <c r="D5" t="str">
-        <v>C</v>
-      </c>
-      <c r="E5">
-        <v>3.3</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Pass</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Mock Data 5</v>
-      </c>
-      <c r="B6">
-        <v>83039</v>
-      </c>
-      <c r="C6" s="1">
-        <v>60415</v>
-      </c>
-      <c r="D6" t="str">
-        <v>B+</v>
-      </c>
-      <c r="E6">
-        <v>2.2</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Pass</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
I have my website deployed in github and when saving the notice.xlsx fil
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,9 +420,43 @@
         <v>details</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Mock Data 3</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2082-11-04</v>
+      </c>
+      <c r="C2" t="str">
+        <v>…</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Calendar</v>
+      </c>
+      <c r="E2" t="str">
+        <v>MockData 1 detailed description …</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Annuals Fo</v>
+      </c>
+      <c r="B3" t="str">
+        <v>387293</v>
+      </c>
+      <c r="C3" t="str">
+        <v>3987</v>
+      </c>
+      <c r="D3" t="str">
+        <v>dc</v>
+      </c>
+      <c r="E3" t="str">
+        <v>3279872</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Is it possible or not:?
I will place this file in a different gitub rep
</commit_message>
<xml_diff>
--- a/public/data/notice.xlsx
+++ b/public/data/notice.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,26 +437,9 @@
         <v>MockData 1 detailed description …</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Annuals Fo</v>
-      </c>
-      <c r="B3" t="str">
-        <v>387293</v>
-      </c>
-      <c r="C3" t="str">
-        <v>3987</v>
-      </c>
-      <c r="D3" t="str">
-        <v>dc</v>
-      </c>
-      <c r="E3" t="str">
-        <v>3279872</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>